<commit_message>
Double-click Full Screen button starts wallboard rotation, same as Ctrl+R
</commit_message>
<xml_diff>
--- a/gridline_import_template.xlsx
+++ b/gridline_import_template.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="0" activeTab="6" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
@@ -16,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Section" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -34,7 +33,7 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="001F3B57"/>
+      <color rgb="FF1F3B57"/>
       <sz val="14"/>
     </font>
     <font>
@@ -44,25 +43,25 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="001F3B57"/>
+      <color rgb="FF1F3B57"/>
       <sz val="11.5"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00A8420C"/>
+      <color rgb="FFA8420C"/>
       <sz val="10.5"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="10.5"/>
     </font>
     <font>
       <name val="Arial"/>
       <i val="1"/>
-      <color rgb="007A5C00"/>
+      <color rgb="FF7A5C00"/>
       <sz val="10.5"/>
     </font>
     <font>
@@ -80,14 +79,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3B57"/>
-        <bgColor rgb="001F3B57"/>
+        <fgColor rgb="FF1F3B57"/>
+        <bgColor rgb="FF1F3B57"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF6CC"/>
-        <bgColor rgb="00FFF6CC"/>
+        <fgColor rgb="FFFFF6CC"/>
+        <bgColor rgb="FFFFF6CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -101,17 +100,18 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D0D5DA"/>
+        <color rgb="FFD0D5DA"/>
       </left>
       <right style="thin">
-        <color rgb="00D0D5DA"/>
+        <color rgb="FFD0D5DA"/>
       </right>
       <top style="thin">
-        <color rgb="00D0D5DA"/>
+        <color rgb="FFD0D5DA"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D0D5DA"/>
+        <color rgb="FFD0D5DA"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -136,7 +136,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -499,29 +499,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A44"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:A57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="18" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>GRIDLINE Network Import Template</t>
         </is>
       </c>
     </row>
-    <row r="2"/>
-    <row r="3">
+    <row r="3" ht="27.5" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Fill in the sheets below with your distribution network, then use “↪ Import Excel” in GRIDLINE to load it. The network will render on the canvas immediately so you can review it before it goes live.</t>
         </is>
       </c>
     </row>
-    <row r="4"/>
-    <row r="5">
+    <row r="5" ht="15" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Where this can be imported</t>
@@ -549,8 +547,7 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
-    <row r="10">
+    <row r="10" ht="15" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Sheets in this workbook</t>
@@ -599,8 +596,7 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
-    <row r="18">
+    <row r="18" ht="15" customHeight="1">
       <c r="A18" s="3" t="inlineStr">
         <is>
           <t>How the Lines sheet works</t>
@@ -664,7 +660,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="inlineStr"/>
+      <c r="A27" s="4" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -695,7 +691,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="inlineStr"/>
+      <c r="A32" s="4" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -718,44 +714,129 @@
         </is>
       </c>
     </row>
-    <row r="36"/>
+    <row r="36">
+      <c r="A36" s="9" t="inlineStr">
+        <is>
+          <t>Attaching MORE THAN ONE transformer to the same line: the Lines sheet's "Transformer Connected"</t>
+        </is>
+      </c>
+    </row>
     <row r="37" ht="45" customHeight="1">
       <c r="A37" s="9" t="inlineStr">
         <is>
+          <t>column only holds one name per row. To add a second (or third...) transformer to that same line,</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="9" t="inlineStr">
+        <is>
+          <t>add extra rows on the Transformers sheet instead -- give each its own unique Transformer Name, and</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="9" t="inlineStr">
+        <is>
+          <t>set Attached Line to that line's auto-generated name (see "L1", "L2" numbering above). Any number of</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="15" customHeight="1">
+      <c r="A40" s="9" t="inlineStr">
+        <is>
+          <t>Transformers-sheet rows may share the same Attached Line value; nothing limits it to one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="9" t="inlineStr">
+        <is>
+          <t>Attached Line vs. Attached Breaker (Transformers sheet): Attached Line places a transformer</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="9" t="inlineStr">
+        <is>
+          <t>along a line SPAN itself -- tapped mid-conductor, using the auto-generated "L1", "L2" names above.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="9" t="inlineStr">
+        <is>
+          <t>Attached Breaker instead places it AT a specific junction/switch point, by that junction's label</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="9" t="inlineStr">
+        <is>
+          <t>from the Lines sheet (e.g. "Kangarappady"). This works for ANY junction type, not only RMU -- AB,</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="9" t="inlineStr">
+        <is>
+          <t>RMU, Split, and Tap labels all work equally. Use whichever matches where the transformer</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="9" t="inlineStr">
+        <is>
+          <t>physically sits; each transformer needs exactly one of the two columns filled in, never both.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="9" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="9" t="n"/>
+    </row>
+    <row r="49"/>
+    <row r="50">
+      <c r="A50" s="9" t="inlineStr">
+        <is>
           <t>Note on interlink state: every ring interlink always starts CLOSED when a file is imported, regardless of the Interlinks sheet's “State” column or the Lines sheet's “AB State” for that row -- an interlink has no switch of its own in real life until you mark it Switchable (Yes) on the Interlinks sheet, and even then it only opens afterward, from within the app itself.</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="3" t="inlineStr">
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
         <is>
           <t>Filling this in</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
-        <is>
-          <t>Each sheet already has one example row, shaded yellow, showing a complete, working network (matching the</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Each sheet already has one or more example rows, shaded yellow, showing a complete, working network (matching the</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
         <is>
           <t>example that GRIDLINE itself starts with on a fresh install). Overwrite the example values with your own data,</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="4" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
         <is>
           <t>or add new rows below it — keep the header row and column order exactly as given. Delete the example row once</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
         <is>
           <t>you no longer need it for reference; an empty sheet is fine for anything optional.</t>
         </is>
@@ -773,13 +854,11 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="2" max="3"/>
+    <col width="10" customWidth="1" min="4" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
   </cols>
@@ -852,7 +931,7 @@
           <t>Judgemukku</t>
         </is>
       </c>
-      <c r="G2" s="7" t="inlineStr"/>
+      <c r="G2" s="7" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
@@ -880,8 +959,8 @@
           <t>Closed</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr"/>
-      <c r="G3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="n"/>
+      <c r="G3" s="7" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
@@ -909,7 +988,7 @@
           <t>Closed</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="n"/>
       <c r="G4" s="7" t="inlineStr">
         <is>
           <t>StyleUnion</t>
@@ -947,7 +1026,7 @@
           <t>Suburban</t>
         </is>
       </c>
-      <c r="G5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -980,7 +1059,7 @@
           <t>Townhall</t>
         </is>
       </c>
-      <c r="G6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -1013,7 +1092,7 @@
           <t>Kangarappady</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -1041,8 +1120,8 @@
           <t>Closed</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr"/>
-      <c r="G8" s="7" t="inlineStr"/>
+      <c r="F8" s="7" t="n"/>
+      <c r="G8" s="7" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -1070,8 +1149,8 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr"/>
-      <c r="G9" s="7" t="inlineStr"/>
+      <c r="F9" s="7" t="n"/>
+      <c r="G9" s="7" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1085,7 +1164,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -1157,7 +1236,7 @@
           <t>Waterlogging near Pipeline junction in monsoon</t>
         </is>
       </c>
-      <c r="F2" s="7" t="inlineStr"/>
+      <c r="F2" s="7" t="n"/>
       <c r="G2" s="7" t="inlineStr">
         <is>
           <t>On</t>
@@ -1183,8 +1262,8 @@
           <t>Section Officer, 9847098765</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr"/>
-      <c r="F3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="n"/>
+      <c r="F3" s="7" t="n"/>
       <c r="G3" s="7" t="inlineStr">
         <is>
           <t>On</t>
@@ -1202,17 +1281,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:K4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="5" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="22" customWidth="1" min="11" max="11"/>
@@ -1281,8 +1357,8 @@
           <t>Judgemukku</t>
         </is>
       </c>
-      <c r="B2" s="7" t="inlineStr"/>
-      <c r="C2" s="7" t="inlineStr"/>
+      <c r="B2" s="7" t="n"/>
+      <c r="C2" s="7" t="n"/>
       <c r="D2" s="7" t="n">
         <v>100</v>
       </c>
@@ -1305,8 +1381,8 @@
           <t>2026-07-20 09:00</t>
         </is>
       </c>
-      <c r="J2" s="7" t="inlineStr"/>
-      <c r="K2" s="7" t="inlineStr"/>
+      <c r="J2" s="7" t="n"/>
+      <c r="K2" s="7" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
@@ -1314,7 +1390,7 @@
           <t>Kangarappady Aux TX</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr"/>
+      <c r="B3" s="7" t="n"/>
       <c r="C3" s="7" t="inlineStr">
         <is>
           <t>Kangarappady</t>
@@ -1352,6 +1428,43 @@
           <t>Overload trip</t>
         </is>
       </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Pipeline Aux TX</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="n"/>
+      <c r="D4" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>P-1B</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="H4" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="I4" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-20 09:00</t>
+        </is>
+      </c>
+      <c r="J4" s="7" t="n"/>
+      <c r="K4" s="7" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1365,13 +1478,11 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="2" max="3"/>
+    <col width="12" customWidth="1" min="4" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -1451,7 +1562,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -1515,7 +1626,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
@@ -1553,7 +1664,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>Kakkanad</t>
+          <t>Aluva</t>
         </is>
       </c>
     </row>

</xml_diff>